<commit_message>
test(core): add fixture regeneration script and documentation for case1/case2/case4 xlsx
- Added generate-fixtures.mjs to deterministically regenerate case1_1904_dates.xlsx,
  case2_numeric_identifiers.xlsx, and case4_complex_sheet.xlsx test fixtures.
- Added README.md documenting the fixture shapes and regeneration commands.
- Verified all real-world fixture test suites pass against the rebuilt files.
</commit_message>
<xml_diff>
--- a/packages/core/test-fixtures/case1_1904_dates.xlsx
+++ b/packages/core/test-fixtures/case1_1904_dates.xlsx
@@ -1,36 +1,49 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr date1904="1"/>
-  <workbookProtection/>
-  <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
-  </bookViews>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr date1904="1" defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Employees" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet sheetId="1" name="Employees" state="visible" r:id="rId4"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>BirthDate</t>
+  </si>
+  <si>
+    <t>JoinDate</t>
+  </si>
+  <si>
+    <t>Alice Mac</t>
+  </si>
+  <si>
+    <t>Bob Mac</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-  </numFmts>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
+      <color theme="1"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+      <sz val="11"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -49,81 +62,22 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -202,6 +156,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -236,6 +191,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -270,20 +226,16 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:shade val="51000"/>
+                <a:tint val="100000"/>
+                <a:shade val="100000"/>
                 <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="80000">
-              <a:schemeClr val="phClr">
-                <a:shade val="93000"/>
-                <a:satMod val="130000"/>
-              </a:schemeClr>
-            </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="94000"/>
-                <a:satMod val="135000"/>
+                <a:tint val="50000"/>
+                <a:shade val="100000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -405,64 +357,90 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
+  <a:objectDefaults>
+    <a:spDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="3">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </a:style>
+    </a:spDef>
+    <a:lnDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </a:style>
+    </a:lnDef>
+  </a:objectDefaults>
   <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Name</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>BirthDate</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>JoinDate</t>
-        </is>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Alice Mac</t>
-        </is>
-      </c>
-      <c r="B2" s="1" t="n">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="1">
         <v>44695</v>
       </c>
-      <c r="C2" s="1" t="n">
+      <c r="C2" s="1">
         <v>1</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Bob Mac</t>
-        </is>
-      </c>
-      <c r="B3" s="1" t="n">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="1">
         <v>29884</v>
       </c>
-      <c r="C3" s="1" t="n">
+      <c r="C3" s="1">
         <v>42429</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
</xml_diff>